<commit_message>
fixed checklist Completed B002 (Gigardos
</commit_message>
<xml_diff>
--- a/SpectrobesSFM checklist.xlsx
+++ b/SpectrobesSFM checklist.xlsx
@@ -14,12 +14,15 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$F$225</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="426">
   <si>
     <t>ID</t>
   </si>
@@ -2139,10 +2142,16 @@
       <c r="B6" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="10"/>
+      <c r="C6" s="65" t="s">
+        <v>424</v>
+      </c>
+      <c r="D6" s="66" t="s">
+        <v>424</v>
+      </c>
+      <c r="E6" s="46"/>
+      <c r="F6" s="67" t="s">
+        <v>424</v>
+      </c>
     </row>
     <row r="7" spans="1:6" ht="12.75">
       <c r="A7" s="5" t="s">

</xml_diff>

<commit_message>
Finished B008 (Jado) and B009 (Terragon)
</commit_message>
<xml_diff>
--- a/SpectrobesSFM checklist.xlsx
+++ b/SpectrobesSFM checklist.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="426">
   <si>
     <t>ID</t>
   </si>
@@ -1699,7 +1699,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1842,6 +1842,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2227,10 +2233,16 @@
       <c r="B10" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="10"/>
+      <c r="C10" s="72" t="s">
+        <v>424</v>
+      </c>
+      <c r="D10" s="73" t="s">
+        <v>424</v>
+      </c>
+      <c r="E10" s="70"/>
+      <c r="F10" s="71" t="s">
+        <v>424</v>
+      </c>
     </row>
     <row r="11" spans="1:6" ht="12.75">
       <c r="A11" s="5" t="s">

</xml_diff>